<commit_message>
Checklist de revisão manual finalizado
- Itens de repositório (R22 a R25) validados, com evidência
- Remove arquivo temporário do Excel versionado por engano e ignora ~$* no .gitignore
</commit_message>
<xml_diff>
--- a/docs/checklist-revisao.xlsx
+++ b/docs/checklist-revisao.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="E:\TesteVerzel\docs\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{46F24693-9E62-4F37-9CAD-8A328ECCD86B}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{3BCCB275-D71C-470E-B307-5859834E5F94}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-120" yWindow="-120" windowWidth="26040" windowHeight="15840" activeTab="1" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -18,14 +18,14 @@
     <sheet name="Resumo" sheetId="3" r:id="rId3"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="1" hidden="1">Checklist!$A$1:$K$27</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="1" hidden="1">Checklist!$A$1:$J$26</definedName>
   </definedNames>
   <calcPr calcId="191029"/>
 </workbook>
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="271" uniqueCount="216">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="276" uniqueCount="218">
   <si>
     <t>Checklist de revisão manual: teste técnico QA Júnior Verzel</t>
   </si>
@@ -534,9 +534,6 @@
     <t>Em uma pasta nova: git clone do repositório, npm install, npx playwright install chromium, npm test.</t>
   </si>
   <si>
-    <t>39 passed (6 deles marcados como falha esperada, com "x" na listagem).</t>
-  </si>
-  <si>
     <t>R23</t>
   </si>
   <si>
@@ -580,18 +577,6 @@
   </si>
   <si>
     <t>79 cenários: 59 ✅ · 13 ❌ · 6 ⚠️ · 1 N/A.</t>
-  </si>
-  <si>
-    <t>R26</t>
-  </si>
-  <si>
-    <t>Seção "Uso de IA" com texto seu</t>
-  </si>
-  <si>
-    <t>Reescrever a seção "Uso de IA" com suas palavras, de forma coerente com o que você vai declarar no formulário de envio.</t>
-  </si>
-  <si>
-    <t>Texto final revisado por você e igual em espírito ao do formulário.</t>
   </si>
   <si>
     <t>Resumo do checklist</t>
@@ -695,6 +680,9 @@
     <t>evidencias\manual\R19.jpg</t>
   </si>
   <si>
+    <t>evidencias\manual\R22.jpg</t>
+  </si>
+  <si>
     <t>Os valores se mantém com 2 casas decimais</t>
   </si>
   <si>
@@ -707,6 +695,24 @@
   </si>
   <si>
     <t>Todos os campos do formulário são devidamente tratados na inserção de dados</t>
+  </si>
+  <si>
+    <t>40 passed (6 deles marcados como falha esperada, com "x" na listagem).</t>
+  </si>
+  <si>
+    <t>40 testes passando e 6 falham como no planejado</t>
+  </si>
+  <si>
+    <t>Todos os links abrem o arquivo ou seção correta, para facilitar revisão posterior</t>
+  </si>
+  <si>
+    <t>N/A</t>
+  </si>
+  <si>
+    <t>Os prints dos bugs condizem com os relatos</t>
+  </si>
+  <si>
+    <t>O total contabilizado no resumo reflete exatamente os dados encontrados nas execuções</t>
   </si>
 </sst>
 </file>
@@ -1312,7 +1318,7 @@
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0100-000000000000}">
-  <dimension ref="A1:K27"/>
+  <dimension ref="A1:J26"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="1" max="1" width="6" customWidth="1"/>
@@ -1325,10 +1331,9 @@
     <col min="8" max="8" width="15" customWidth="1"/>
     <col min="9" max="9" width="28" customWidth="1"/>
     <col min="10" max="10" width="12" customWidth="1"/>
-    <col min="11" max="11" width="35" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:11" ht="30" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="1" spans="1:10" ht="30" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A1" s="5" t="s">
         <v>26</v>
       </c>
@@ -1359,11 +1364,8 @@
       <c r="J1" s="5" t="s">
         <v>22</v>
       </c>
-      <c r="K1" s="5" t="s">
-        <v>24</v>
-      </c>
-    </row>
-    <row r="2" spans="1:11" ht="75" customHeight="1" x14ac:dyDescent="0.25">
+    </row>
+    <row r="2" spans="1:10" ht="75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A2" s="6" t="s">
         <v>32</v>
       </c>
@@ -1394,9 +1396,8 @@
       <c r="J2" s="8">
         <v>46302</v>
       </c>
-      <c r="K2" s="7"/>
-    </row>
-    <row r="3" spans="1:11" ht="60" customHeight="1" x14ac:dyDescent="0.25">
+    </row>
+    <row r="3" spans="1:10" ht="60" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A3" s="6" t="s">
         <v>40</v>
       </c>
@@ -1427,9 +1428,8 @@
       <c r="J3" s="8">
         <v>46302</v>
       </c>
-      <c r="K3" s="7"/>
-    </row>
-    <row r="4" spans="1:11" ht="30" customHeight="1" x14ac:dyDescent="0.25">
+    </row>
+    <row r="4" spans="1:10" ht="30" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A4" s="6" t="s">
         <v>47</v>
       </c>
@@ -1460,9 +1460,8 @@
       <c r="J4" s="8">
         <v>46302</v>
       </c>
-      <c r="K4" s="7"/>
-    </row>
-    <row r="5" spans="1:11" ht="90" customHeight="1" x14ac:dyDescent="0.25">
+    </row>
+    <row r="5" spans="1:10" ht="90" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A5" s="6" t="s">
         <v>54</v>
       </c>
@@ -1493,9 +1492,8 @@
       <c r="J5" s="8">
         <v>46302</v>
       </c>
-      <c r="K5" s="7"/>
-    </row>
-    <row r="6" spans="1:11" ht="120" customHeight="1" x14ac:dyDescent="0.25">
+    </row>
+    <row r="6" spans="1:10" ht="120" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A6" s="6" t="s">
         <v>61</v>
       </c>
@@ -1526,9 +1524,8 @@
       <c r="J6" s="8">
         <v>46302</v>
       </c>
-      <c r="K6" s="7"/>
-    </row>
-    <row r="7" spans="1:11" ht="30" customHeight="1" x14ac:dyDescent="0.25">
+    </row>
+    <row r="7" spans="1:10" ht="30" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A7" s="6" t="s">
         <v>67</v>
       </c>
@@ -1559,9 +1556,8 @@
       <c r="J7" s="8">
         <v>46302</v>
       </c>
-      <c r="K7" s="7"/>
-    </row>
-    <row r="8" spans="1:11" ht="79.5" customHeight="1" x14ac:dyDescent="0.25">
+    </row>
+    <row r="8" spans="1:10" ht="79.5" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A8" s="6" t="s">
         <v>74</v>
       </c>
@@ -1592,9 +1588,8 @@
       <c r="J8" s="8">
         <v>46302</v>
       </c>
-      <c r="K8" s="7"/>
-    </row>
-    <row r="9" spans="1:11" ht="45" customHeight="1" x14ac:dyDescent="0.25">
+    </row>
+    <row r="9" spans="1:10" ht="45" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A9" s="6" t="s">
         <v>82</v>
       </c>
@@ -1625,9 +1620,8 @@
       <c r="J9" s="8">
         <v>46302</v>
       </c>
-      <c r="K9" s="7"/>
-    </row>
-    <row r="10" spans="1:11" ht="159.94999999999999" customHeight="1" x14ac:dyDescent="0.25">
+    </row>
+    <row r="10" spans="1:10" ht="159.94999999999999" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A10" s="6" t="s">
         <v>90</v>
       </c>
@@ -1658,9 +1652,8 @@
       <c r="J10" s="8">
         <v>46302</v>
       </c>
-      <c r="K10" s="7"/>
-    </row>
-    <row r="11" spans="1:11" ht="159.94999999999999" customHeight="1" x14ac:dyDescent="0.25">
+    </row>
+    <row r="11" spans="1:10" ht="159.94999999999999" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A11" s="6" t="s">
         <v>97</v>
       </c>
@@ -1674,26 +1667,25 @@
         <v>99</v>
       </c>
       <c r="E11" s="16" t="s">
-        <v>188</v>
+        <v>183</v>
       </c>
       <c r="F11" s="6" t="s">
         <v>100</v>
       </c>
       <c r="G11" s="7" t="s">
-        <v>189</v>
+        <v>184</v>
       </c>
       <c r="H11" s="7" t="s">
         <v>19</v>
       </c>
       <c r="I11" s="7" t="s">
-        <v>190</v>
+        <v>185</v>
       </c>
       <c r="J11" s="8">
         <v>46302</v>
       </c>
-      <c r="K11" s="7"/>
-    </row>
-    <row r="12" spans="1:11" ht="30" customHeight="1" x14ac:dyDescent="0.25">
+    </row>
+    <row r="12" spans="1:10" ht="30" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A12" s="6" t="s">
         <v>101</v>
       </c>
@@ -1713,20 +1705,19 @@
         <v>106</v>
       </c>
       <c r="G12" s="7" t="s">
-        <v>191</v>
+        <v>186</v>
       </c>
       <c r="H12" s="7" t="s">
         <v>19</v>
       </c>
       <c r="I12" s="7" t="s">
-        <v>192</v>
+        <v>187</v>
       </c>
       <c r="J12" s="8">
         <v>46302</v>
       </c>
-      <c r="K12" s="7"/>
-    </row>
-    <row r="13" spans="1:11" ht="30" customHeight="1" x14ac:dyDescent="0.25">
+    </row>
+    <row r="13" spans="1:10" ht="30" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A13" s="6" t="s">
         <v>107</v>
       </c>
@@ -1746,20 +1737,19 @@
         <v>111</v>
       </c>
       <c r="G13" s="7" t="s">
-        <v>194</v>
+        <v>189</v>
       </c>
       <c r="H13" s="7" t="s">
-        <v>197</v>
+        <v>192</v>
       </c>
       <c r="I13" s="7" t="s">
-        <v>195</v>
+        <v>190</v>
       </c>
       <c r="J13" s="8">
         <v>46302</v>
       </c>
-      <c r="K13" s="7"/>
-    </row>
-    <row r="14" spans="1:11" ht="15" customHeight="1" x14ac:dyDescent="0.25">
+    </row>
+    <row r="14" spans="1:10" ht="15" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A14" s="6" t="s">
         <v>112</v>
       </c>
@@ -1779,20 +1769,19 @@
         <v>116</v>
       </c>
       <c r="G14" s="7" t="s">
-        <v>196</v>
+        <v>191</v>
       </c>
       <c r="H14" s="7" t="s">
-        <v>197</v>
+        <v>192</v>
       </c>
       <c r="I14" s="7" t="s">
-        <v>198</v>
+        <v>193</v>
       </c>
       <c r="J14" s="8">
         <v>46302</v>
       </c>
-      <c r="K14" s="7"/>
-    </row>
-    <row r="15" spans="1:11" ht="15" customHeight="1" x14ac:dyDescent="0.25">
+    </row>
+    <row r="15" spans="1:10" ht="15" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A15" s="6" t="s">
         <v>117</v>
       </c>
@@ -1812,20 +1801,19 @@
         <v>121</v>
       </c>
       <c r="G15" s="7" t="s">
-        <v>199</v>
+        <v>194</v>
       </c>
       <c r="H15" s="7" t="s">
-        <v>197</v>
+        <v>192</v>
       </c>
       <c r="I15" s="7" t="s">
-        <v>200</v>
+        <v>195</v>
       </c>
       <c r="J15" s="8">
         <v>46302</v>
       </c>
-      <c r="K15" s="7"/>
-    </row>
-    <row r="16" spans="1:11" ht="30" customHeight="1" x14ac:dyDescent="0.25">
+    </row>
+    <row r="16" spans="1:10" ht="30" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A16" s="6" t="s">
         <v>122</v>
       </c>
@@ -1845,20 +1833,19 @@
         <v>126</v>
       </c>
       <c r="G16" s="7" t="s">
-        <v>201</v>
+        <v>196</v>
       </c>
       <c r="H16" s="7" t="s">
+        <v>192</v>
+      </c>
+      <c r="I16" s="7" t="s">
         <v>197</v>
-      </c>
-      <c r="I16" s="7" t="s">
-        <v>202</v>
       </c>
       <c r="J16" s="8">
         <v>46302</v>
       </c>
-      <c r="K16" s="7"/>
-    </row>
-    <row r="17" spans="1:11" ht="50.25" customHeight="1" x14ac:dyDescent="0.25">
+    </row>
+    <row r="17" spans="1:10" ht="50.25" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A17" s="6" t="s">
         <v>127</v>
       </c>
@@ -1872,26 +1859,25 @@
         <v>129</v>
       </c>
       <c r="E17" s="6" t="s">
-        <v>203</v>
+        <v>198</v>
       </c>
       <c r="F17" s="6" t="s">
-        <v>204</v>
+        <v>199</v>
       </c>
       <c r="G17" s="7" t="s">
-        <v>205</v>
+        <v>200</v>
       </c>
       <c r="H17" s="7" t="s">
-        <v>197</v>
+        <v>192</v>
       </c>
       <c r="I17" s="7" t="s">
-        <v>206</v>
+        <v>201</v>
       </c>
       <c r="J17" s="8">
         <v>46302</v>
       </c>
-      <c r="K17" s="7"/>
-    </row>
-    <row r="18" spans="1:11" ht="30" customHeight="1" x14ac:dyDescent="0.25">
+    </row>
+    <row r="18" spans="1:10" ht="30" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A18" s="6" t="s">
         <v>130</v>
       </c>
@@ -1911,20 +1897,19 @@
         <v>134</v>
       </c>
       <c r="G18" s="7" t="s">
-        <v>207</v>
+        <v>202</v>
       </c>
       <c r="H18" s="7" t="s">
-        <v>197</v>
+        <v>192</v>
       </c>
       <c r="I18" s="7" t="s">
-        <v>208</v>
+        <v>203</v>
       </c>
       <c r="J18" s="8">
         <v>46302</v>
       </c>
-      <c r="K18" s="7"/>
-    </row>
-    <row r="19" spans="1:11" ht="101.25" customHeight="1" x14ac:dyDescent="0.25">
+    </row>
+    <row r="19" spans="1:10" ht="101.25" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A19" s="6" t="s">
         <v>135</v>
       </c>
@@ -1944,20 +1929,19 @@
         <v>139</v>
       </c>
       <c r="G19" s="7" t="s">
-        <v>209</v>
+        <v>204</v>
       </c>
       <c r="H19" s="7" t="s">
-        <v>197</v>
+        <v>192</v>
       </c>
       <c r="I19" s="7" t="s">
-        <v>210</v>
+        <v>205</v>
       </c>
       <c r="J19" s="8">
         <v>46302</v>
       </c>
-      <c r="K19" s="7"/>
-    </row>
-    <row r="20" spans="1:11" ht="30" customHeight="1" x14ac:dyDescent="0.25">
+    </row>
+    <row r="20" spans="1:10" ht="30" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A20" s="6" t="s">
         <v>140</v>
       </c>
@@ -1977,20 +1961,19 @@
         <v>144</v>
       </c>
       <c r="G20" s="7" t="s">
-        <v>212</v>
+        <v>208</v>
       </c>
       <c r="H20" s="7" t="s">
-        <v>197</v>
+        <v>192</v>
       </c>
       <c r="I20" s="7" t="s">
-        <v>211</v>
+        <v>206</v>
       </c>
       <c r="J20" s="8">
         <v>46302</v>
       </c>
-      <c r="K20" s="7"/>
-    </row>
-    <row r="21" spans="1:11" ht="105.75" customHeight="1" x14ac:dyDescent="0.25">
+    </row>
+    <row r="21" spans="1:10" ht="105.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A21" s="6" t="s">
         <v>145</v>
       </c>
@@ -2010,20 +1993,19 @@
         <v>150</v>
       </c>
       <c r="G21" s="7" t="s">
-        <v>213</v>
+        <v>209</v>
       </c>
       <c r="H21" s="7" t="s">
-        <v>197</v>
+        <v>192</v>
       </c>
       <c r="I21" s="7" t="s">
-        <v>214</v>
+        <v>210</v>
       </c>
       <c r="J21" s="8">
         <v>46302</v>
       </c>
-      <c r="K21" s="7"/>
-    </row>
-    <row r="22" spans="1:11" ht="30" customHeight="1" x14ac:dyDescent="0.25">
+    </row>
+    <row r="22" spans="1:10" ht="30" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A22" s="6" t="s">
         <v>151</v>
       </c>
@@ -2043,20 +2025,19 @@
         <v>155</v>
       </c>
       <c r="G22" s="7" t="s">
-        <v>215</v>
+        <v>211</v>
       </c>
       <c r="H22" s="7" t="s">
-        <v>197</v>
+        <v>192</v>
       </c>
       <c r="I22" s="7" t="s">
-        <v>193</v>
+        <v>188</v>
       </c>
       <c r="J22" s="8">
         <v>46302</v>
       </c>
-      <c r="K22" s="7"/>
-    </row>
-    <row r="23" spans="1:11" ht="30" customHeight="1" x14ac:dyDescent="0.25">
+    </row>
+    <row r="23" spans="1:10" ht="30" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A23" s="6" t="s">
         <v>156</v>
       </c>
@@ -2073,127 +2054,120 @@
         <v>160</v>
       </c>
       <c r="F23" s="6" t="s">
-        <v>161</v>
-      </c>
-      <c r="G23" s="7"/>
-      <c r="H23" s="7"/>
-      <c r="I23" s="7"/>
+        <v>212</v>
+      </c>
+      <c r="G23" s="7" t="s">
+        <v>213</v>
+      </c>
+      <c r="H23" s="7" t="s">
+        <v>192</v>
+      </c>
+      <c r="I23" s="7" t="s">
+        <v>207</v>
+      </c>
       <c r="J23" s="8">
         <v>46302</v>
       </c>
-      <c r="K23" s="7"/>
-    </row>
-    <row r="24" spans="1:11" ht="45" customHeight="1" x14ac:dyDescent="0.25">
+    </row>
+    <row r="24" spans="1:10" ht="45" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A24" s="6" t="s">
-        <v>162</v>
+        <v>161</v>
       </c>
       <c r="B24" s="6" t="s">
         <v>157</v>
       </c>
       <c r="C24" s="6" t="s">
+        <v>162</v>
+      </c>
+      <c r="D24" s="6" t="s">
         <v>163</v>
       </c>
-      <c r="D24" s="6" t="s">
+      <c r="E24" s="6" t="s">
         <v>164</v>
       </c>
-      <c r="E24" s="6" t="s">
+      <c r="F24" s="6" t="s">
         <v>165</v>
       </c>
-      <c r="F24" s="6" t="s">
-        <v>166</v>
-      </c>
-      <c r="G24" s="7"/>
-      <c r="H24" s="7"/>
-      <c r="I24" s="7"/>
+      <c r="G24" s="7" t="s">
+        <v>214</v>
+      </c>
+      <c r="H24" s="7" t="s">
+        <v>192</v>
+      </c>
+      <c r="I24" s="7" t="s">
+        <v>215</v>
+      </c>
       <c r="J24" s="8">
         <v>46302</v>
       </c>
-      <c r="K24" s="7"/>
-    </row>
-    <row r="25" spans="1:11" ht="30" customHeight="1" x14ac:dyDescent="0.25">
+    </row>
+    <row r="25" spans="1:10" ht="30" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A25" s="6" t="s">
-        <v>167</v>
+        <v>166</v>
       </c>
       <c r="B25" s="6" t="s">
         <v>157</v>
       </c>
       <c r="C25" s="6" t="s">
+        <v>167</v>
+      </c>
+      <c r="D25" s="6" t="s">
         <v>168</v>
       </c>
-      <c r="D25" s="6" t="s">
+      <c r="E25" s="6" t="s">
         <v>169</v>
       </c>
-      <c r="E25" s="6" t="s">
+      <c r="F25" s="6" t="s">
         <v>170</v>
       </c>
-      <c r="F25" s="6" t="s">
-        <v>171</v>
-      </c>
-      <c r="G25" s="7"/>
-      <c r="H25" s="7"/>
-      <c r="I25" s="7"/>
+      <c r="G25" s="7" t="s">
+        <v>216</v>
+      </c>
+      <c r="H25" s="7" t="s">
+        <v>192</v>
+      </c>
+      <c r="I25" s="7" t="s">
+        <v>215</v>
+      </c>
       <c r="J25" s="8">
         <v>46302</v>
       </c>
-      <c r="K25" s="7"/>
-    </row>
-    <row r="26" spans="1:11" ht="30" customHeight="1" x14ac:dyDescent="0.25">
+    </row>
+    <row r="26" spans="1:10" ht="57.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A26" s="6" t="s">
-        <v>172</v>
+        <v>171</v>
       </c>
       <c r="B26" s="6" t="s">
         <v>157</v>
       </c>
       <c r="C26" s="6" t="s">
+        <v>172</v>
+      </c>
+      <c r="D26" s="6" t="s">
         <v>173</v>
       </c>
-      <c r="D26" s="6" t="s">
+      <c r="E26" s="6" t="s">
         <v>174</v>
       </c>
-      <c r="E26" s="6" t="s">
+      <c r="F26" s="6" t="s">
         <v>175</v>
       </c>
-      <c r="F26" s="6" t="s">
-        <v>176</v>
-      </c>
-      <c r="G26" s="7"/>
-      <c r="H26" s="7"/>
-      <c r="I26" s="7"/>
+      <c r="G26" s="7" t="s">
+        <v>217</v>
+      </c>
+      <c r="H26" s="7" t="s">
+        <v>192</v>
+      </c>
+      <c r="I26" s="7" t="s">
+        <v>215</v>
+      </c>
       <c r="J26" s="8">
         <v>46302</v>
       </c>
-      <c r="K26" s="7"/>
-    </row>
-    <row r="27" spans="1:11" ht="30" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A27" s="6" t="s">
-        <v>177</v>
-      </c>
-      <c r="B27" s="6" t="s">
-        <v>157</v>
-      </c>
-      <c r="C27" s="6" t="s">
-        <v>158</v>
-      </c>
-      <c r="D27" s="6" t="s">
-        <v>178</v>
-      </c>
-      <c r="E27" s="6" t="s">
-        <v>179</v>
-      </c>
-      <c r="F27" s="6" t="s">
-        <v>180</v>
-      </c>
-      <c r="G27" s="7"/>
-      <c r="H27" s="7"/>
-      <c r="I27" s="7"/>
-      <c r="J27" s="8">
-        <v>46302</v>
-      </c>
-      <c r="K27" s="7"/>
     </row>
   </sheetData>
-  <autoFilter ref="A1:K27" xr:uid="{00000000-0009-0000-0000-000001000000}"/>
-  <conditionalFormatting sqref="H2:H27">
+  <autoFilter ref="A1:J26" xr:uid="{00000000-0009-0000-0000-000001000000}"/>
+  <conditionalFormatting sqref="H2:H26">
     <cfRule type="expression" dxfId="2" priority="1">
       <formula>$H2="OK"</formula>
     </cfRule>
@@ -2205,7 +2179,7 @@
     </cfRule>
   </conditionalFormatting>
   <dataValidations count="1">
-    <dataValidation type="list" allowBlank="1" errorTitle="Status inválido" error="Escolha OK, Divergente ou Não executado." sqref="H2:H27" xr:uid="{00000000-0002-0000-0100-000000000000}">
+    <dataValidation type="list" allowBlank="1" errorTitle="Status inválido" error="Escolha OK, Divergente ou Não executado." sqref="H2:H26" xr:uid="{00000000-0002-0000-0100-000000000000}">
       <formula1>"OK,Divergente,Não executado"</formula1>
     </dataValidation>
   </dataValidations>
@@ -2225,7 +2199,7 @@
   <sheetData>
     <row r="2" spans="2:7" ht="16.5" customHeight="1" x14ac:dyDescent="0.25">
       <c r="B2" s="9" t="s">
-        <v>181</v>
+        <v>176</v>
       </c>
     </row>
     <row r="4" spans="2:7" x14ac:dyDescent="0.25">
@@ -2233,19 +2207,19 @@
         <v>27</v>
       </c>
       <c r="C4" s="10" t="s">
-        <v>182</v>
+        <v>177</v>
       </c>
       <c r="D4" s="10" t="s">
         <v>19</v>
       </c>
       <c r="E4" s="10" t="s">
-        <v>183</v>
+        <v>178</v>
       </c>
       <c r="F4" s="10" t="s">
-        <v>184</v>
+        <v>179</v>
       </c>
       <c r="G4" s="10" t="s">
-        <v>185</v>
+        <v>180</v>
       </c>
     </row>
     <row r="5" spans="2:7" x14ac:dyDescent="0.25">
@@ -2253,19 +2227,19 @@
         <v>33</v>
       </c>
       <c r="C5" s="12">
-        <f>COUNTIF(Checklist!$B$2:$B$27,B5)</f>
+        <f>COUNTIF(Checklist!$B$2:$B$26,B5)</f>
         <v>7</v>
       </c>
       <c r="D5" s="12">
-        <f>COUNTIFS(Checklist!$B$2:$B$27,B5,Checklist!$H$2:$H$27,"OK")</f>
+        <f>COUNTIFS(Checklist!$B$2:$B$26,B5,Checklist!$H$2:$H$26,"OK")</f>
         <v>7</v>
       </c>
       <c r="E5" s="12">
-        <f>COUNTIFS(Checklist!$B$2:$B$27,B5,Checklist!$H$2:$H$27,"Divergente")</f>
+        <f>COUNTIFS(Checklist!$B$2:$B$26,B5,Checklist!$H$2:$H$26,"Divergente")</f>
         <v>0</v>
       </c>
       <c r="F5" s="12">
-        <f>COUNTIFS(Checklist!$B$2:$B$27,B5,Checklist!$H$2:$H$27,"Não executado")</f>
+        <f>COUNTIFS(Checklist!$B$2:$B$26,B5,Checklist!$H$2:$H$26,"Não executado")</f>
         <v>0</v>
       </c>
       <c r="G5" s="12">
@@ -2278,19 +2252,19 @@
         <v>75</v>
       </c>
       <c r="C6" s="12">
-        <f>COUNTIF(Checklist!$B$2:$B$27,B6)</f>
+        <f>COUNTIF(Checklist!$B$2:$B$26,B6)</f>
         <v>2</v>
       </c>
       <c r="D6" s="12">
-        <f>COUNTIFS(Checklist!$B$2:$B$27,B6,Checklist!$H$2:$H$27,"OK")</f>
+        <f>COUNTIFS(Checklist!$B$2:$B$26,B6,Checklist!$H$2:$H$26,"OK")</f>
         <v>2</v>
       </c>
       <c r="E6" s="12">
-        <f>COUNTIFS(Checklist!$B$2:$B$27,B6,Checklist!$H$2:$H$27,"Divergente")</f>
+        <f>COUNTIFS(Checklist!$B$2:$B$26,B6,Checklist!$H$2:$H$26,"Divergente")</f>
         <v>0</v>
       </c>
       <c r="F6" s="12">
-        <f>COUNTIFS(Checklist!$B$2:$B$27,B6,Checklist!$H$2:$H$27,"Não executado")</f>
+        <f>COUNTIFS(Checklist!$B$2:$B$26,B6,Checklist!$H$2:$H$26,"Não executado")</f>
         <v>0</v>
       </c>
       <c r="G6" s="12">
@@ -2303,19 +2277,19 @@
         <v>83</v>
       </c>
       <c r="C7" s="12">
-        <f>COUNTIF(Checklist!$B$2:$B$27,B7)</f>
+        <f>COUNTIF(Checklist!$B$2:$B$26,B7)</f>
         <v>1</v>
       </c>
       <c r="D7" s="12">
-        <f>COUNTIFS(Checklist!$B$2:$B$27,B7,Checklist!$H$2:$H$27,"OK")</f>
+        <f>COUNTIFS(Checklist!$B$2:$B$26,B7,Checklist!$H$2:$H$26,"OK")</f>
         <v>1</v>
       </c>
       <c r="E7" s="12">
-        <f>COUNTIFS(Checklist!$B$2:$B$27,B7,Checklist!$H$2:$H$27,"Divergente")</f>
+        <f>COUNTIFS(Checklist!$B$2:$B$26,B7,Checklist!$H$2:$H$26,"Divergente")</f>
         <v>0</v>
       </c>
       <c r="F7" s="12">
-        <f>COUNTIFS(Checklist!$B$2:$B$27,B7,Checklist!$H$2:$H$27,"Não executado")</f>
+        <f>COUNTIFS(Checklist!$B$2:$B$26,B7,Checklist!$H$2:$H$26,"Não executado")</f>
         <v>0</v>
       </c>
       <c r="G7" s="12">
@@ -2328,19 +2302,19 @@
         <v>102</v>
       </c>
       <c r="C8" s="12">
-        <f>COUNTIF(Checklist!$B$2:$B$27,B8)</f>
+        <f>COUNTIF(Checklist!$B$2:$B$26,B8)</f>
         <v>9</v>
       </c>
       <c r="D8" s="12">
-        <f>COUNTIFS(Checklist!$B$2:$B$27,B8,Checklist!$H$2:$H$27,"OK")</f>
+        <f>COUNTIFS(Checklist!$B$2:$B$26,B8,Checklist!$H$2:$H$26,"OK")</f>
         <v>9</v>
       </c>
       <c r="E8" s="12">
-        <f>COUNTIFS(Checklist!$B$2:$B$27,B8,Checklist!$H$2:$H$27,"Divergente")</f>
+        <f>COUNTIFS(Checklist!$B$2:$B$26,B8,Checklist!$H$2:$H$26,"Divergente")</f>
         <v>0</v>
       </c>
       <c r="F8" s="12">
-        <f>COUNTIFS(Checklist!$B$2:$B$27,B8,Checklist!$H$2:$H$27,"Não executado")</f>
+        <f>COUNTIFS(Checklist!$B$2:$B$26,B8,Checklist!$H$2:$H$26,"Não executado")</f>
         <v>0</v>
       </c>
       <c r="G8" s="12">
@@ -2353,19 +2327,19 @@
         <v>146</v>
       </c>
       <c r="C9" s="12">
-        <f>COUNTIF(Checklist!$B$2:$B$27,B9)</f>
+        <f>COUNTIF(Checklist!$B$2:$B$26,B9)</f>
         <v>2</v>
       </c>
       <c r="D9" s="12">
-        <f>COUNTIFS(Checklist!$B$2:$B$27,B9,Checklist!$H$2:$H$27,"OK")</f>
+        <f>COUNTIFS(Checklist!$B$2:$B$26,B9,Checklist!$H$2:$H$26,"OK")</f>
         <v>2</v>
       </c>
       <c r="E9" s="12">
-        <f>COUNTIFS(Checklist!$B$2:$B$27,B9,Checklist!$H$2:$H$27,"Divergente")</f>
+        <f>COUNTIFS(Checklist!$B$2:$B$26,B9,Checklist!$H$2:$H$26,"Divergente")</f>
         <v>0</v>
       </c>
       <c r="F9" s="12">
-        <f>COUNTIFS(Checklist!$B$2:$B$27,B9,Checklist!$H$2:$H$27,"Não executado")</f>
+        <f>COUNTIFS(Checklist!$B$2:$B$26,B9,Checklist!$H$2:$H$26,"Não executado")</f>
         <v>0</v>
       </c>
       <c r="G9" s="12">
@@ -2378,37 +2352,37 @@
         <v>157</v>
       </c>
       <c r="C10" s="12">
-        <f>COUNTIF(Checklist!$B$2:$B$27,B10)</f>
-        <v>5</v>
+        <f>COUNTIF(Checklist!$B$2:$B$26,B10)</f>
+        <v>4</v>
       </c>
       <c r="D10" s="12">
-        <f>COUNTIFS(Checklist!$B$2:$B$27,B10,Checklist!$H$2:$H$27,"OK")</f>
+        <f>COUNTIFS(Checklist!$B$2:$B$26,B10,Checklist!$H$2:$H$26,"OK")</f>
+        <v>4</v>
+      </c>
+      <c r="E10" s="12">
+        <f>COUNTIFS(Checklist!$B$2:$B$26,B10,Checklist!$H$2:$H$26,"Divergente")</f>
         <v>0</v>
       </c>
-      <c r="E10" s="12">
-        <f>COUNTIFS(Checklist!$B$2:$B$27,B10,Checklist!$H$2:$H$27,"Divergente")</f>
-        <v>0</v>
-      </c>
       <c r="F10" s="12">
-        <f>COUNTIFS(Checklist!$B$2:$B$27,B10,Checklist!$H$2:$H$27,"Não executado")</f>
+        <f>COUNTIFS(Checklist!$B$2:$B$26,B10,Checklist!$H$2:$H$26,"Não executado")</f>
         <v>0</v>
       </c>
       <c r="G10" s="12">
         <f t="shared" si="0"/>
-        <v>5</v>
+        <v>0</v>
       </c>
     </row>
     <row r="11" spans="2:7" x14ac:dyDescent="0.25">
       <c r="B11" s="13" t="s">
-        <v>186</v>
+        <v>181</v>
       </c>
       <c r="C11" s="14">
         <f>SUM(C5:C10)</f>
-        <v>26</v>
+        <v>25</v>
       </c>
       <c r="D11" s="14">
         <f>SUM(D5:D10)</f>
-        <v>21</v>
+        <v>25</v>
       </c>
       <c r="E11" s="14">
         <f>SUM(E5:E10)</f>
@@ -2420,12 +2394,12 @@
       </c>
       <c r="G11" s="14">
         <f>SUM(G5:G10)</f>
-        <v>5</v>
+        <v>0</v>
       </c>
     </row>
     <row r="13" spans="2:7" x14ac:dyDescent="0.25">
       <c r="B13" s="15" t="s">
-        <v>187</v>
+        <v>182</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Verificação final: sintaxe Gherkin, print de erro de roteiro e datas do checklist
- carrinho.feature: passo "Quando, mesmo assim," não era reconhecido pelo parser Gherkin
- Remove CT-CAR-03-erro.png, sobra de uma falha do roteiro (não da loja)
- Datas da revisão manual atualizadas no checklist
</commit_message>
<xml_diff>
--- a/docs/checklist-revisao.xlsx
+++ b/docs/checklist-revisao.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="E:\TesteVerzel\docs\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{C69A787D-02FA-47B4-AADC-DA7D80306E59}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{9423FC29-3E7B-4F97-B98C-BDA9A7A2A793}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-120" yWindow="-120" windowWidth="26040" windowHeight="15840" activeTab="1" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -1970,7 +1970,7 @@
         <v>166</v>
       </c>
       <c r="J20" s="8">
-        <v>46302</v>
+        <v>46303</v>
       </c>
     </row>
     <row r="21" spans="1:10" ht="105.75" customHeight="1" x14ac:dyDescent="0.25">

</xml_diff>

<commit_message>
Checklist R22: prints do clone em pasta nova e da execução (40 aprovados)
</commit_message>
<xml_diff>
--- a/docs/checklist-revisao.xlsx
+++ b/docs/checklist-revisao.xlsx
@@ -1932,11 +1932,11 @@
       </c>
       <c r="I23" s="7" t="inlineStr">
         <is>
-          <t>evidencias\manual\R22.jpg</t>
+          <t>evidencias\manual\R22-clone.png e evidencias\manual\R22-execucao.png</t>
         </is>
       </c>
       <c r="J23" s="8" t="n">
-        <v>46302</v>
+        <v>46304</v>
       </c>
     </row>
     <row r="24" ht="45" customHeight="1" s="18">

</xml_diff>

<commit_message>
Detalhes da revisão: asserções em todos os ramos do CT-QTD-07 e /api/ no BUG-03
- CT-QTD-07: ramos de bloqueio verificam aviso de limite ou quantidade ajustada
- CT-API-05 cobre /api e /api/; nova evidência CT-API-05-b.json (404 JSON)
- BUG-03 com análise (hipótese) e sugestão; R07 do checklist inclui curl de /api/
</commit_message>
<xml_diff>
--- a/docs/checklist-revisao.xlsx
+++ b/docs/checklist-revisao.xlsx
@@ -1139,13 +1139,15 @@
       </c>
       <c r="E8" s="6" t="inlineStr">
         <is>
-          <t>No terminal: curl -i https://verzel-store.qa-test-verzel-store.workers.dev/api
-Depois: curl -i https://verzel-store.qa-test-verzel-store.workers.dev/api/rota-inexistente</t>
+          <t>No terminal:
+curl -i https://verzel-store.qa-test-verzel-store.workers.dev/api
+curl -i https://verzel-store.qa-test-verzel-store.workers.dev/api/
+curl -i https://verzel-store.qa-test-verzel-store.workers.dev/api/rota-inexistente</t>
         </is>
       </c>
       <c r="F8" s="6" t="inlineStr">
         <is>
-          <t>Registrado: /api → 200 com Content-Type text/html; /api/rota-inexistente → 404 JSON ROTA_NAO_ENCONTRADA.</t>
+          <t>Registrado: /api → 200 com Content-Type text/html; /api/ (com barra) e /api/rota-inexistente → 404 JSON ROTA_NAO_ENCONTRADA.</t>
         </is>
       </c>
       <c r="G8" s="7" t="inlineStr">

</xml_diff>